<commit_message>
correct column J header to C3
</commit_message>
<xml_diff>
--- a/input_data/flow_scen/FallFlows20261021_Draft.xlsx
+++ b/input_data/flow_scen/FallFlows20261021_Draft.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/lelliott_usbr_gov/Documents/Documents/GitHub/BDO-Science/Fall_Flow_Redd_Dewatering/input_data/flow_scen/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="8_{E7DFD7F7-14B9-49AC-881D-4D1AA1487E0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{78A3519B-7038-40A6-AE78-2F0138ADA956}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="8_{E7DFD7F7-14B9-49AC-881D-4D1AA1487E0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D4DE55A-7F58-411E-B2B0-10A7CFA736B9}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="876" xr2:uid="{8B6B0201-DD1B-4D0A-8FA2-1793C828B1EC}"/>
   </bookViews>
@@ -1960,19 +1960,19 @@
                   <c:v>-100</c:v>
                 </c:pt>
                 <c:pt idx="81">
-                  <c:v>10000000</c:v>
+                  <c:v>-100</c:v>
                 </c:pt>
                 <c:pt idx="82">
-                  <c:v>10000000</c:v>
+                  <c:v>-100</c:v>
                 </c:pt>
                 <c:pt idx="83">
-                  <c:v>10000000</c:v>
+                  <c:v>-100</c:v>
                 </c:pt>
                 <c:pt idx="84">
-                  <c:v>10000000</c:v>
+                  <c:v>-100</c:v>
                 </c:pt>
                 <c:pt idx="85">
-                  <c:v>10000000</c:v>
+                  <c:v>-100</c:v>
                 </c:pt>
                 <c:pt idx="86">
                   <c:v>10000000</c:v>
@@ -13047,7 +13047,7 @@
         <v>55</v>
       </c>
       <c r="J2" s="13" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="K2" s="13"/>
       <c r="L2" s="13"/>
@@ -15856,7 +15856,7 @@
       <c r="O84" s="10"/>
       <c r="P84">
         <f t="shared" ca="1" si="2"/>
-        <v>10000000</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="85" spans="1:16" x14ac:dyDescent="0.3">
@@ -15896,7 +15896,7 @@
       <c r="O85" s="10"/>
       <c r="P85">
         <f t="shared" ca="1" si="2"/>
-        <v>10000000</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="86" spans="1:16" x14ac:dyDescent="0.3">
@@ -15936,7 +15936,7 @@
       <c r="O86" s="10"/>
       <c r="P86">
         <f t="shared" ca="1" si="2"/>
-        <v>10000000</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="87" spans="1:16" x14ac:dyDescent="0.3">
@@ -15976,7 +15976,7 @@
       <c r="O87" s="10"/>
       <c r="P87">
         <f t="shared" ca="1" si="2"/>
-        <v>10000000</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="88" spans="1:16" x14ac:dyDescent="0.3">
@@ -16016,7 +16016,7 @@
       <c r="O88" s="10"/>
       <c r="P88">
         <f t="shared" ca="1" si="2"/>
-        <v>10000000</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="89" spans="1:16" x14ac:dyDescent="0.3">
@@ -16047,7 +16047,7 @@
         <v>6500</v>
       </c>
       <c r="J89" s="10">
-        <v>5500</v>
+        <v>6000</v>
       </c>
       <c r="K89" s="1"/>
       <c r="L89" s="1"/>
@@ -21198,7 +21198,7 @@
       </c>
       <c r="J219" s="15">
         <f t="shared" si="15"/>
-        <v>5903.2258064516127</v>
+        <v>5919.3548387096771</v>
       </c>
       <c r="K219" s="15" t="e">
         <f>AVERAGE(K64:K94)</f>
@@ -21571,7 +21571,7 @@
       </c>
       <c r="J227" s="15">
         <f t="shared" si="39"/>
-        <v>362.97501</v>
+        <v>363.966745</v>
       </c>
       <c r="K227" s="15" t="e">
         <f>((1.98347*31)*K219)/1000</f>
@@ -21844,7 +21844,7 @@
       </c>
       <c r="J232" s="51">
         <f t="shared" si="58"/>
-        <v>1752.15574513</v>
+        <v>1753.1474801300001</v>
       </c>
       <c r="K232" s="51" t="e">
         <f t="shared" si="57"/>
@@ -21898,7 +21898,7 @@
       </c>
       <c r="J233" s="51">
         <f t="shared" ref="J233" si="60">SUM(J226:J228)</f>
-        <v>1038.1065451300001</v>
+        <v>1039.0982801299999</v>
       </c>
       <c r="K233" s="51" t="e">
         <f t="shared" si="59"/>

</xml_diff>